<commit_message>
Data Driven Testing - 2
</commit_message>
<xml_diff>
--- a/seleniumproject/testdata/loginData.xlsx
+++ b/seleniumproject/testdata/loginData.xlsx
@@ -8,16 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\D Drive\seleniumproject\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E82DA3E-197F-43AC-B893-3D51A5C8CC4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C0D17783-F1BA-4A40-B8C9-79684027E5F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{911BE987-616B-404A-9753-44586D822034}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{776D5C5C-31C4-4696-9B05-73869FD062CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
-    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
-    <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="9">
   <si>
     <t>Username</t>
   </si>
@@ -46,41 +42,48 @@
     <t>Password</t>
   </si>
   <si>
-    <t>admin123</t>
-  </si>
-  <si>
-    <t>Role</t>
-  </si>
-  <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>Tester</t>
-  </si>
-  <si>
-    <t>User</t>
-  </si>
-  <si>
-    <t>test123</t>
-  </si>
-  <si>
-    <t>user123</t>
-  </si>
-  <si>
-    <t>Customer</t>
+    <t>standard_user</t>
+  </si>
+  <si>
+    <t>locked_out_user</t>
+  </si>
+  <si>
+    <t>problem_user</t>
+  </si>
+  <si>
+    <t>performance_glitch_user</t>
+  </si>
+  <si>
+    <t>error_user</t>
+  </si>
+  <si>
+    <t>visual_user</t>
+  </si>
+  <si>
+    <t>secret_sauce</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -103,8 +106,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -418,95 +423,71 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FED5F3D7-71D8-4BA2-8BC4-56CB21DBEE97}">
-  <dimension ref="A1:C4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{578E3C92-4E64-42A5-80C6-C2592927CCE2}">
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.88671875" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="1" max="1" width="35.88671875" customWidth="1"/>
+    <col min="2" max="2" width="36.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
+      <c r="B7" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B493A2B2-991B-49FC-ABBA-44BB7F5E44F0}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71943053-EB47-4EC5-817C-F136131026FD}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB59279B-7CD2-4088-B60A-999C1D2B4CA5}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ADABFCF-7DD7-4BC5-98B9-A7FCC858E2DE}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>